<commit_message>
chore: update news radar report 2026-10-07
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-10-07.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-10-07.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -477,27 +477,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mark Cuban's Cost-Plus Enters New Jersey Employer Benefits Market</t>
+          <t>Manufacturers Launch 340B Rebate Pilot Programs</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Mark Cuban Cost Plus Drug Company is expanding its pharmacy benefits model into New Jersey's employer market, intensifying competition against traditional PBMs. This move offers self-funded employers alternative pricing structures focused on transparency and direct-to-consumer cost savings. The entry signals continued disruption in the PBM space as employers seek non-traditional partners to manage rising drug expenditures.</t>
+          <t>Pharmaceutical manufacturers are rolling out new 340B rebate pilot initiatives, shifting how covered entities and contract pharmacies manage pricing. This development impacts drug distribution channels and overall program integrity, which heavily influence pharmacy benefit management and commercial health plan costs.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BenefitsPRO</t>
+          <t>JDSupra</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Tue, 06 Oct 2026 15:24:27 GMT</t>
+          <t>Wed, 07 Oct 2026 15:37:05 GMT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOMHNxZVo2SWd0N3FxcEN3UnVad3ZMZDNFQ3B1aTZxYTRRblJBcThKU1MycUVjMG56OXowR0RZalpGS2txeDlGZG01RmYxZGxIVEhacXF6RXpjZEM1Y0cySUJHTWc4aDkwN3JrdVdScHY0YkFKcUFXWndKSUFSLUNzMjlfbjZnRnIxamE4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPRXRPVmNYbU9zWElmaERGck1VOHh4MHp2Y2diMU52YjJBcy0xTUxxV3gyendyLVphUTNrbnd5R3pCdnkzbUltclFYWmRMaXdmLW5MQlVIekhxUGJSM0VQY3RuMjB5WkpWN2RSM0JlcHJGVUJURGJ4SmUtLXhwVThwZFZfNEswZ0xH?oc=5</t>
         </is>
       </c>
     </row>
@@ -507,27 +507,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Insurer-Owned PBMs Lose Ground in Commercial Health Plan Market</t>
+          <t>Gross-to-Net Realities Highlight Evolving Drug Channel Pricing Dynamics</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Insurer-owned pharmacy benefit managers are experiencing a decline in market share within the commercial sector as employers increasingly seek alternatives. This shift highlights growing employer dissatisfaction with traditional integrated PBM models and creates opportunities for independent, transparent PBM alternatives.</t>
+          <t>An analysis of 2025 gross-to-net pricing data from top drugmakers examines the shifting dynamics of the net pricing drug channel. This data is critical for self-funded employers and PBMs evaluating net versus gross drug spend and rebate structures. Understanding these trends helps plan sponsors better manage escalating specialty and brand drug costs.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BenefitsPRO</t>
+          <t>Drug Channels</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Tue, 06 Oct 2026 15:24:27 GMT</t>
+          <t>Wed, 07 Oct 2026 09:30:00 GMT</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxPTkxOYzlFWlFJd1NqdzVvVDdQMXQyWUJoU2FZMHRzYzlGVXpqRC14WlVfN0FNbUM4Q0pETlkzM2dQSDFiWmVHM05uR0N5QWlMb2NRVXZDRzh1U2FsdkRfeGVySy04OHRRaUktTXBUR0pURnpmUnRPdVNib1lGUUR2NENOdWdwdEdRNVc5eFdmeXIyTkhZdENTTHh0bS0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQY05yRHRQaWYtZ0hKc29heDEtb05aMEcwQXp0bzJ1Q3A4RkdDOFlLcGJQM0NGV1Z6ZkFDejJuVWFMbE13SDZubUxhcC1SbUVPV0hOSENVRDhJMThRTHNTbFg4cU8xRjB5RWptcmh3NE9SX3dMTnVocEJobm9vNXY1Z0VCZ0E?oc=5</t>
         </is>
       </c>
     </row>
@@ -537,27 +537,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Rebates Rise While Self-Funded Pharmacy Costs Climb</t>
+          <t>Rising Pharmacy Benefit Rebates Fail to Curb Climbing Employer Drug Costs</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The article examines the disconnect between increasing pharmaceutical manufacturer rebates and the ongoing rise in overall employer-sponsored pharmacy plan costs. This dynamic directly impacts self-funded employers struggling to manage net drug spend despite traditional PBM rebate guarantees. The key implication is that employers must look beyond headline rebates and scrutinize underlying pricing structures and PBM alignment to truly control specialty and total pharmacy expenditures.</t>
+          <t>As pharmacy benefit rebates continue to rise, self-funded employers report that overall drug costs keep climbing unabated. This trend underscores ongoing frustrations with PBM pricing transparency and net versus gross drug spend management. The dynamic reinforces the strategic importance for employers to evaluate transparent, pass-through PBM models to capture true savings.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Insurance Business</t>
+          <t>Human Resources Director</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Tue, 06 Oct 2026 11:07:24 GMT</t>
+          <t>Wed, 07 Oct 2026 01:40:14 GMT</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQbkdwWTdpcTZlX0w4ZnVld18wRXVPa2pkcmo1VHFCZ3VzcklXZTdKVkpMZUZKQmNrOFctaXBvOFBMbF9qUFc0aVhnSGlNNGFtVUE0aFFNU050SVRLZGVVbVVhX2Nmc1BOSHBnekxLdXVEdkRIMGtEdTVDTjNJRVVsRzFweUFQVjhPY1RLQnUwRU12ZDYzNUxDZWlFSmlRa3gyMVZoTUdoMXJFNFNrS2NMcFVZTXVXMmM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQY0F0MnVvNWdqVEFyODRWU2c5SXpkUlREM21oQ0oyYkhrZWNmSzRIWXF0LTI5aHF5UGhlV0lLekpfV0c2S3lGNjhwWElyNGYtajZ1Y3JkS2Y0R2R4dkREdDdYcDl5cVJuTFRKZ0RRUDB5X3RPQWJsR29vbkh4aURWYW5HVE1GdlE5aDRZNm8tTnpqTVEtZmU3T2FFa3hwcWhtQXdpVTZ1bEVxWnFWTUYyalVHU1VLakhjUUZINFRlOTA?oc=5</t>
         </is>
       </c>
     </row>
@@ -567,27 +567,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Congressional PBM Reform Faces Hurdles Before Reaching Consumers</t>
+          <t>PBM Transparency Gaps Challenge Employer Cost-Containment Efforts</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>The article discusses ongoing legislative efforts surrounding pharmacy benefit manager (PBM) reform and the challenges Congress faces in passing impactful measures that directly benefit consumers and plan sponsors. This is strategically important for self-funded employers and PBMs monitoring federal policy shifts, transparency demands, and potential regulatory changes to drug pricing models.</t>
+          <t>Despite ongoing regulatory scrutiny, pharmacy benefit managers continue to maintain opaque pricing practices that make it difficult for self-funded employers to control drug spend. The article examines actionable strategies for plan sponsors to demand greater contract clarity and rein in rising pharmacy costs.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>ProMarket</t>
+          <t>MedCity News</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Tue, 06 Oct 2026 10:00:00 GMT</t>
+          <t>Wed, 07 Oct 2026 13:45:52 GMT</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNdHdiRVo1U3dMWnNDVnIxckNHWjlMNjBCemVqUkhXNVh3R08zZkdudl9HNDBHSGN0cnFmQ3RVano0WFUtRU1STk53MG80NTNWSldoeFQta1lxcVN4aDV3eHFlOEpOTmg3UGhtbkF0R2VxbkFVLXpKdE9id0Z6UjVOVDBJczFNa0hqZUVNb09qUUk5enE1cFBIYXJ5VEdza2xibFNMbQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxON0UxQ0U3a3kyOVlDdjhVNVZxeFFqZUNNVjJ3cGQ1ckpNeHhMOU5kdnVlbUZQZUNTNXlMblFBMFlrSGN3Ul8xdmhZTFdTSnpiVVNqUGdSYnpUZTB1bHdiZ0c0cDhHWHBWRUVQT0g3QWRCRU1GclB0N0djX3kxUEJSblpZWmJBc0Q5bWIyVTlfaXYzUWRNR3RpVFNzSWxydmVjZllPV1lXN3ZIdw?oc=5</t>
         </is>
       </c>
     </row>
@@ -597,27 +597,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Optum Rx and Express Scripts Extend Market Lead Over Rival PBMs</t>
+          <t>Congress Targets PBM and Broker Payments Amid Employer Drug Market Shifts</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Recent data highlights that Optum Rx and Express Scripts have further cemented their dominant market share positions within the pharmacy benefit management industry. This consolidation of power among the largest PBMs impacts the competitive landscape for self-funded employers seeking alternatives for transparent, cost-effective benefit management.</t>
+          <t>Lawmakers are increasingly scrutinizing financial arrangements between pharmacy benefit managers and brokers, focusing on how hidden fees impact self-funded employer health plan costs. This legislative attention signals potential regulatory changes for employer drug benefit distribution and transparency.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Modern Healthcare</t>
+          <t>Insurance Business</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Tue, 06 Oct 2026 16:00:00 GMT</t>
+          <t>Wed, 07 Oct 2026 11:07:25 GMT</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxNbkdlcnkyQ2JOMFNIZDAxUnVWSkI5X012NnVMbVBXV3o2WkZCeE1jWk13bzRyWU53VjBBM2pMeTlRaE4xZW9CdndxenJTaDhBQS05SzZORXc0dklMU3BUUXJYbWhTaW40akh5Z2FrRjZBTy1sVTk1SDJuT2p5ckVKUGJLUE9EUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQbkZtNkh0U19Sb3J0MXBVV29qZ0xvbERVMS1OMzMzLW94eFR2UDVqYW16OGxEMlNkSGY3Nzh0bHdaRlhVVEpCM2NuNDFBX1JBeHdUX1VWYVRMamtLU0xuWXlITV9mbGd6bWdqX2V0OUstNlFiMndfaVJ6MWlra3VzdnhrSjRNR3ExUFY3NFhya2FPY3JIRWpCZXdEY1pFeXVWd3hwTWRkZjNhcFhDWElDeUdVUzhxZEJBLWpWelJxOF9RdndEZmpIVlc5Ylo?oc=5</t>
         </is>
       </c>
     </row>
@@ -627,27 +627,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Judge Stays Public Nuisance Lawsuit Against Major PBMs</t>
+          <t>Clarventa Launches TrueNet to Reshape Prescription Drug Pricing Models</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>A federal judge has agreed to stay a public nuisance case targeting major pharmacy benefit managers. This litigation pause impacts ongoing legal challenges surrounding PBM business practices and pricing models, which are of high strategic interest to self-funded employers monitoring industry accountability.</t>
+          <t>Clarventa has announced TrueNet, a novel approach aimed at reforming prescription drug pricing and transparency for self-funded health plans. This launch reflects ongoing market pressure for alternative pricing models that challenge traditional PBM structures. The development is strategically important for employers seeking greater transparency and cost predictability in their pharmacy benefits.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Mealey's</t>
+          <t>Business Wire</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Tue, 06 Oct 2026 17:56:54 GMT</t>
+          <t>Wed, 07 Oct 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQR0xYRU1BaXJwZG9WM01TRTlhSG5ZT3MxRW4tQ0VIbmtTNS1qMzhEa0E1dkhtRjJYUnNIcnl5Wnc3aU56blVTaC14SlBpb3pRa1cxM0ZrUV92ZUV1cjNoMGpFT1Ztdm9yV21SZm43TlkwUVpPM2JNeGZtalJrTVotQW5QZmVKQUVjSlZ3SS1tN2tsUUlXMDU2ZHc0VmplelNNdXhaVGJkemVVMFpuRzU1c2JacXhKbGtGZzFJT3ZBOWRfdWhQS0JocnNLOHFMcW0wbVNyTjI4T2p0TlpZTHpaQdIBYkFVX3lxTE5PTkNpM2E0cUdtenhpYVJ6ZXNUcTEwb0lXaXgyRnRvQnRUYTBmT3kwdkxhT3JUWFZleWp3TjBHQVM2SmFNNGwyS0RQVFJ0SURSbFBnNHpoS1p2dDNJMERtbmtn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOZTRNNldGeEk5TmJRUExCeHhFU1JuWUVVc1RfX1ZOa1pNR1NuS051b3U0dURSUk5xRFZ1RkNZT3J4bGNZd3g3MEhnOEY1T09BWm1Wa0h1OHBOTElWeGE5a1A0YkxaaUt5NUR2TzBiLVIxMFpINm5qZG5BOGhsaXBlaWRHUTZCWTZmNG5HbXJJQ0tTaHYwTDkxV1M4eGpHU1lxQ0gtd1dNNElMOFIxbHdKcVh2eFRTem8zbHhZcjV1LTdacGh0ejd3?oc=5</t>
         </is>
       </c>
     </row>
@@ -657,117 +657,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Rewriting the Post-Exclusivity Playbook for Generics and Biosimilars</t>
+          <t>Virta Health Reaches Profitability Amid Growing Employer Adoption</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>The article examines how the pharmaceutical market is evolving post-exclusivity for major drugs, focusing on strategies for generics and biosimilars. This is critically important for self-funded employers and PBMs looking to leverage biosimilar adoption and generic competition to drive down surging specialty and prescription drug costs. The implication is a shifting formulary landscape that requires active management to maximize savings from upcoming patent cliffs.</t>
+          <t>Virta Health announced it has reached profitability and now serves over 750 organizations, highlighting strong employer demand for digital health solutions targeting chronic conditions like type 2 diabetes. This growth reflects how self-funded employers are increasingly partnering with specialized point solutions to manage high-cost metabolic diseases and potentially offset soaring pharmacy spend. The milestone underscores the expanding market for integrated chronic disease management within employer-sponsored health plans.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>PharmaLive</t>
+          <t>Lelezard</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Tue, 06 Oct 2026 13:49:30 GMT</t>
+          <t>Wed, 07 Oct 2026 04:36:32 GMT</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQVjA5eXJFOTBkMFBDSHc2WXNDSTdpMk9WbHpXZDM1SVUwWXBWQjh1b21GMXFFWEt1Qk9LbENfMmZvUkltZnVBd1dwS2s5a1V5djlJeEdhem1TWlZSamxGVDcxaFBTYzhkdmw5UXBmR3A4QTRaWHNsR1NuZHd6YmdYYV80TE1TRkx5em12VXRhRVhFTzRwcWRoUU9MZHBic1ZETEhFYjZUUDNNWXNtUTdJRlVueU9zY0MxbkpnUG4wZHVVQQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>McKesson and CD&amp;R Acquire Option Care Health for $5.8 Billion</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>McKesson and Clayton, Dubilier &amp; Rice have agreed to acquire infusion services provider Option Care Health in a $5.8 billion deal. This major consolidation in specialty healthcare impacts the specialty pharmacy landscape, which is critical for self-funded employers managing high-cost specialty drug spend.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Bloomberg.com</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 06 Oct 2026 12:14:43 GMT</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNcms0dzBodUZnQlJNS042X0s5WkF0Q2lwS0VDOENsQlJNeHJad3VNcEpOSjJ2aFFtVWQzX1pkTVlVUDBHbWYtSXdTSWd2SmQ3OHI4SmI4WVRxUUFUczNTQml4TFliTFI5UnZDYnd4WXA4T2otN1hWTDF5M25XeWV6a0NTLUJ2UGJpS295dHVjSHdUdlFBRF9oc3Jsd2FNVVIzTWhaVDh1OExSMl95Nmpn?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>PharmaForce Launches Connected 340B Rebate and MFP Solution</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>PharmaForce has introduced an integrated solution designed to manage 340B rebates and the Maximum Fair Price (MFP) program. This technology impacts drug pricing operations and compliance within the pharmacy supply chain, which directly affects PBM operations and stakeholder cost management.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Business Wire</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 06 Oct 2026 18:03:00 GMT</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNU2dzOUNHRWdIcThNOXNoNG4xNVlFaWFGcXE3Wi1iQ1dGR0lBZVVaX2hncVN3MV9MOU9scEhIWDRBX1lGUUhiaUktWV93YXNFVlF1Q0tRc0o3UXk0OFNCNFlXZUY5c0UwcGg0OGFNTnl6bFUtUW1KUmpTQmRLckJsYUxKU042bU1yYU9LYzhXY09rQy1rV1laRUpFd19YbXo4MnU3dXQydFBzR3lmM1p4SHE0UEhJdw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Rising Hospital and Drug Costs Threaten Self-Funded Employer Health Plans</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Soaring medical and pharmaceutical prices are placing an unsustainable financial burden on American businesses sponsoring self-funded health plans. The pressure highlights the urgent need for employers to implement aggressive cost-management strategies and PBM transparency measures.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Word &amp; Brown General Agency</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 06 Oct 2026 17:05:21 GMT</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQZ2xweWQtZXdRVElNVWd4dGx3TlItdEhaZHVkbVBJRlVOckRNSlp0d1duTW9GWHFKaWdETjNWTkI0RlpTLXF1TFVkUlNaM0ZHa3ZheUFfWUNFTHBlcjFQZmRmemxiT016QmpycmRvWHFKZFJqYmoxQjJpb1NHb2FQQ2JCb2thUzJCS2RKQkJaaXJxQmk1VXA1NWtidlRfd2hQbi1ZeWozeXctUmIyNnpVT0FSai0zUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOOGVYem9ZdU1vdmhBNlRkTUZvU2NPQWFhblgzWG5VbHdDNXBVcUtvQWVVZldqY2Zjb2IzeWFRS1hvT0h2TjVvZU5IMGQtNHJzUDJmM3R3S2NIeEJEV0RybFV4OGwzZGdjdnJpc0pxNkNKU0lUb1ctUC02ZWVUcU1samFDWVJkZ25rSUM3Wk9WM0FuQXlwcmRibkJnWFR6aHFzMzZpRWFsck93S1pNVkc4ZERuRUhVYW41d1BQdVJn?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>